<commit_message>
Update model, analysis functions, notebooks, and results
</commit_message>
<xml_diff>
--- a/M_smegmatis_O2/Experimental_data.xlsx
+++ b/M_smegmatis_O2/Experimental_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/02ff00bc61bfec36/DAE Model Analysis/DAE_System_Model_Calibration_and_Validation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/02ff00bc61bfec36/DAE Model Analysis/DAE_System_Model_Calibration_and_Validation/M_smegmatis_O2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_9595CCCB5F96CA554F11C8179BBD7EA587F59ABE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_9595CCCB5F96CA554F11C8179BBD7EA587F59ABE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA2F0700-629D-4A30-80AE-8CD557E2B9BE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2100" yWindow="3960" windowWidth="21600" windowHeight="13185" tabRatio="870" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PE_Normal" sheetId="1" r:id="rId1"/>
@@ -4625,7 +4625,7 @@
         <v>3.3333333333335586E-3</v>
       </c>
       <c r="J7" s="5">
-        <f t="shared" si="0"/>
+        <f>10^-G7</f>
         <v>0.99990884569276095</v>
       </c>
     </row>

</xml_diff>